<commit_message>
Add Colab · T4 GPU results (t4gpu)
</commit_message>
<xml_diff>
--- a/results/Week05_Benchmark_Workbook.xlsx
+++ b/results/Week05_Benchmark_Workbook.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Board" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Methodology" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Acc_Runs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Latency_Runs" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ScalingLaw" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Hardware" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Board" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VM_vs_GPU" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acc_Runs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latency_Runs" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ScalingLaw" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hardware" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -174,28 +175,28 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>13</row>
+      <row>22</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7677150" cy="5695950"/>
+    <ext cx="15354300" cy="5695950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -492,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -528,7 +529,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>[cpu] Intel VM (CPU only) | 13th Gen Intel(R) Core(TM) i9-13900HX | torch 2.14.1+cpu | seeds [0, 1, 2] | 5 trials x 300 timed forwards, batch 1, n_test=2000</t>
+          <t>[cpu] Intel VM (CPU only) | 13th Gen Intel(R) Core(TM) i9-13900HX | torch 2.14.1+cpu | seeds [0, 1, 2] | 5 trials x 300 timed forwards, batch 1, n_test=2000   ||   [t4gpu] Colab (T4 GPU) | Tesla T4 | torch 2.11.0+cu130 | seeds [0, 1, 2] | 5 trials x 300 timed forwards, batch 1, n_test=2000</t>
         </is>
       </c>
     </row>
@@ -672,25 +673,25 @@
         <v>0.5427</v>
       </c>
       <c r="H5" s="3">
-        <f>AVERAGEIFS(Acc_Runs!D2:D22,Acc_Runs!A2:A22,A5,Acc_Runs!B2:B22,B5)</f>
+        <f>AVERAGEIFS(Acc_Runs!D2:D49,Acc_Runs!A2:A49,A5,Acc_Runs!B2:B49,B5)</f>
         <v/>
       </c>
       <c r="I5" s="3" t="n">
         <v>0.01261942946412397</v>
       </c>
       <c r="J5" s="3">
-        <f>AVERAGEIFS(Acc_Runs!F2:F22,Acc_Runs!A2:A22,A5,Acc_Runs!B2:B22,B5)</f>
+        <f>AVERAGEIFS(Acc_Runs!F2:F49,Acc_Runs!A2:A49,A5,Acc_Runs!B2:B49,B5)</f>
         <v/>
       </c>
       <c r="K5" s="4">
-        <f>AVERAGEIFS(Latency_Runs!E2:E36,Latency_Runs!A2:A36,A5,Latency_Runs!B2:B36,B5)</f>
+        <f>AVERAGEIFS(Latency_Runs!E2:E81,Latency_Runs!A2:A81,A5,Latency_Runs!B2:B81,B5)</f>
         <v/>
       </c>
       <c r="L5" s="4" t="n">
         <v>0.006994158842332671</v>
       </c>
       <c r="M5" s="4">
-        <f>AVERAGEIFS(Latency_Runs!F2:F36,Latency_Runs!A2:A36,A5,Latency_Runs!B2:B36,B5)</f>
+        <f>AVERAGEIFS(Latency_Runs!F2:F81,Latency_Runs!A2:A81,A5,Latency_Runs!B2:B81,B5)</f>
         <v/>
       </c>
       <c r="N5" s="4" t="n">
@@ -746,25 +747,25 @@
         <v>0.5427</v>
       </c>
       <c r="H6" s="3">
-        <f>AVERAGEIFS(Acc_Runs!D2:D22,Acc_Runs!A2:A22,A6,Acc_Runs!B2:B22,B6)</f>
+        <f>AVERAGEIFS(Acc_Runs!D2:D49,Acc_Runs!A2:A49,A6,Acc_Runs!B2:B49,B6)</f>
         <v/>
       </c>
       <c r="I6" s="3" t="n">
         <v>0.01252996408614168</v>
       </c>
       <c r="J6" s="3">
-        <f>AVERAGEIFS(Acc_Runs!F2:F22,Acc_Runs!A2:A22,A6,Acc_Runs!B2:B22,B6)</f>
+        <f>AVERAGEIFS(Acc_Runs!F2:F49,Acc_Runs!A2:A49,A6,Acc_Runs!B2:B49,B6)</f>
         <v/>
       </c>
       <c r="K6" s="4">
-        <f>AVERAGEIFS(Latency_Runs!E2:E36,Latency_Runs!A2:A36,A6,Latency_Runs!B2:B36,B6)</f>
+        <f>AVERAGEIFS(Latency_Runs!E2:E81,Latency_Runs!A2:A81,A6,Latency_Runs!B2:B81,B6)</f>
         <v/>
       </c>
       <c r="L6" s="4" t="n">
         <v>0.01374806292794725</v>
       </c>
       <c r="M6" s="4">
-        <f>AVERAGEIFS(Latency_Runs!F2:F36,Latency_Runs!A2:A36,A6,Latency_Runs!B2:B36,B6)</f>
+        <f>AVERAGEIFS(Latency_Runs!F2:F81,Latency_Runs!A2:A81,A6,Latency_Runs!B2:B81,B6)</f>
         <v/>
       </c>
       <c r="N6" s="4" t="n">
@@ -829,25 +830,25 @@
         <v>0.4471</v>
       </c>
       <c r="H7" s="3">
-        <f>AVERAGEIFS(Acc_Runs!D2:D22,Acc_Runs!A2:A22,A7,Acc_Runs!B2:B22,B7)</f>
+        <f>AVERAGEIFS(Acc_Runs!D2:D49,Acc_Runs!A2:A49,A7,Acc_Runs!B2:B49,B7)</f>
         <v/>
       </c>
       <c r="I7" s="3" t="n">
         <v>0.008621678104251716</v>
       </c>
       <c r="J7" s="3">
-        <f>AVERAGEIFS(Acc_Runs!F2:F22,Acc_Runs!A2:A22,A7,Acc_Runs!B2:B22,B7)</f>
+        <f>AVERAGEIFS(Acc_Runs!F2:F49,Acc_Runs!A2:A49,A7,Acc_Runs!B2:B49,B7)</f>
         <v/>
       </c>
       <c r="K7" s="4">
-        <f>AVERAGEIFS(Latency_Runs!E2:E36,Latency_Runs!A2:A36,A7,Latency_Runs!B2:B36,B7)</f>
+        <f>AVERAGEIFS(Latency_Runs!E2:E81,Latency_Runs!A2:A81,A7,Latency_Runs!B2:B81,B7)</f>
         <v/>
       </c>
       <c r="L7" s="4" t="n">
         <v>0.005299929808446431</v>
       </c>
       <c r="M7" s="4">
-        <f>AVERAGEIFS(Latency_Runs!F2:F36,Latency_Runs!A2:A36,A7,Latency_Runs!B2:B36,B7)</f>
+        <f>AVERAGEIFS(Latency_Runs!F2:F81,Latency_Runs!A2:A81,A7,Latency_Runs!B2:B81,B7)</f>
         <v/>
       </c>
       <c r="N7" s="4" t="n">
@@ -912,25 +913,25 @@
         <v>0.4471</v>
       </c>
       <c r="H8" s="3">
-        <f>AVERAGEIFS(Acc_Runs!D2:D22,Acc_Runs!A2:A22,A8,Acc_Runs!B2:B22,B8)</f>
+        <f>AVERAGEIFS(Acc_Runs!D2:D49,Acc_Runs!A2:A49,A8,Acc_Runs!B2:B49,B8)</f>
         <v/>
       </c>
       <c r="I8" s="3" t="n">
         <v>0.01381122731693312</v>
       </c>
       <c r="J8" s="3">
-        <f>AVERAGEIFS(Acc_Runs!F2:F22,Acc_Runs!A2:A22,A8,Acc_Runs!B2:B22,B8)</f>
+        <f>AVERAGEIFS(Acc_Runs!F2:F49,Acc_Runs!A2:A49,A8,Acc_Runs!B2:B49,B8)</f>
         <v/>
       </c>
       <c r="K8" s="4">
-        <f>AVERAGEIFS(Latency_Runs!E2:E36,Latency_Runs!A2:A36,A8,Latency_Runs!B2:B36,B8)</f>
+        <f>AVERAGEIFS(Latency_Runs!E2:E81,Latency_Runs!A2:A81,A8,Latency_Runs!B2:B81,B8)</f>
         <v/>
       </c>
       <c r="L8" s="4" t="n">
         <v>0.01773631195213339</v>
       </c>
       <c r="M8" s="4">
-        <f>AVERAGEIFS(Latency_Runs!F2:F36,Latency_Runs!A2:A36,A8,Latency_Runs!B2:B36,B8)</f>
+        <f>AVERAGEIFS(Latency_Runs!F2:F81,Latency_Runs!A2:A81,A8,Latency_Runs!B2:B81,B8)</f>
         <v/>
       </c>
       <c r="N8" s="4" t="n">
@@ -995,25 +996,25 @@
         <v>0.0462</v>
       </c>
       <c r="H9" s="3">
-        <f>AVERAGEIFS(Acc_Runs!D2:D22,Acc_Runs!A2:A22,A9,Acc_Runs!B2:B22,B9)</f>
+        <f>AVERAGEIFS(Acc_Runs!D2:D49,Acc_Runs!A2:A49,A9,Acc_Runs!B2:B49,B9)</f>
         <v/>
       </c>
       <c r="I9" s="3" t="n">
         <v>0.009087537253477088</v>
       </c>
       <c r="J9" s="3">
-        <f>AVERAGEIFS(Acc_Runs!F2:F22,Acc_Runs!A2:A22,A9,Acc_Runs!B2:B22,B9)</f>
+        <f>AVERAGEIFS(Acc_Runs!F2:F49,Acc_Runs!A2:A49,A9,Acc_Runs!B2:B49,B9)</f>
         <v/>
       </c>
       <c r="K9" s="4">
-        <f>AVERAGEIFS(Latency_Runs!E2:E36,Latency_Runs!A2:A36,A9,Latency_Runs!B2:B36,B9)</f>
+        <f>AVERAGEIFS(Latency_Runs!E2:E81,Latency_Runs!A2:A81,A9,Latency_Runs!B2:B81,B9)</f>
         <v/>
       </c>
       <c r="L9" s="4" t="n">
         <v>0.01304829515716722</v>
       </c>
       <c r="M9" s="4">
-        <f>AVERAGEIFS(Latency_Runs!F2:F36,Latency_Runs!A2:A36,A9,Latency_Runs!B2:B36,B9)</f>
+        <f>AVERAGEIFS(Latency_Runs!F2:F81,Latency_Runs!A2:A81,A9,Latency_Runs!B2:B81,B9)</f>
         <v/>
       </c>
       <c r="N9" s="4" t="n">
@@ -1078,25 +1079,25 @@
         <v>0.0462</v>
       </c>
       <c r="H10" s="3">
-        <f>AVERAGEIFS(Acc_Runs!D2:D22,Acc_Runs!A2:A22,A10,Acc_Runs!B2:B22,B10)</f>
+        <f>AVERAGEIFS(Acc_Runs!D2:D49,Acc_Runs!A2:A49,A10,Acc_Runs!B2:B49,B10)</f>
         <v/>
       </c>
       <c r="I10" s="3" t="n">
         <v>0.006048415770541379</v>
       </c>
       <c r="J10" s="3">
-        <f>AVERAGEIFS(Acc_Runs!F2:F22,Acc_Runs!A2:A22,A10,Acc_Runs!B2:B22,B10)</f>
+        <f>AVERAGEIFS(Acc_Runs!F2:F49,Acc_Runs!A2:A49,A10,Acc_Runs!B2:B49,B10)</f>
         <v/>
       </c>
       <c r="K10" s="4">
-        <f>AVERAGEIFS(Latency_Runs!E2:E36,Latency_Runs!A2:A36,A10,Latency_Runs!B2:B36,B10)</f>
+        <f>AVERAGEIFS(Latency_Runs!E2:E81,Latency_Runs!A2:A81,A10,Latency_Runs!B2:B81,B10)</f>
         <v/>
       </c>
       <c r="L10" s="4" t="n">
         <v>0.005623055525747161</v>
       </c>
       <c r="M10" s="4">
-        <f>AVERAGEIFS(Latency_Runs!F2:F36,Latency_Runs!A2:A36,A10,Latency_Runs!B2:B36,B10)</f>
+        <f>AVERAGEIFS(Latency_Runs!F2:F81,Latency_Runs!A2:A81,A10,Latency_Runs!B2:B81,B10)</f>
         <v/>
       </c>
       <c r="N10" s="4" t="n">
@@ -1161,25 +1162,25 @@
         <v>0.2439</v>
       </c>
       <c r="H11" s="3">
-        <f>AVERAGEIFS(Acc_Runs!D2:D22,Acc_Runs!A2:A22,A11,Acc_Runs!B2:B22,B11)</f>
+        <f>AVERAGEIFS(Acc_Runs!D2:D49,Acc_Runs!A2:A49,A11,Acc_Runs!B2:B49,B11)</f>
         <v/>
       </c>
       <c r="I11" s="3" t="n">
         <v>0.01307988277215563</v>
       </c>
       <c r="J11" s="3">
-        <f>AVERAGEIFS(Acc_Runs!F2:F22,Acc_Runs!A2:A22,A11,Acc_Runs!B2:B22,B11)</f>
+        <f>AVERAGEIFS(Acc_Runs!F2:F49,Acc_Runs!A2:A49,A11,Acc_Runs!B2:B49,B11)</f>
         <v/>
       </c>
       <c r="K11" s="4">
-        <f>AVERAGEIFS(Latency_Runs!E2:E36,Latency_Runs!A2:A36,A11,Latency_Runs!B2:B36,B11)</f>
+        <f>AVERAGEIFS(Latency_Runs!E2:E81,Latency_Runs!A2:A81,A11,Latency_Runs!B2:B81,B11)</f>
         <v/>
       </c>
       <c r="L11" s="4" t="n">
         <v>0.007886016548185494</v>
       </c>
       <c r="M11" s="4">
-        <f>AVERAGEIFS(Latency_Runs!F2:F36,Latency_Runs!A2:A36,A11,Latency_Runs!B2:B36,B11)</f>
+        <f>AVERAGEIFS(Latency_Runs!F2:F81,Latency_Runs!A2:A81,A11,Latency_Runs!B2:B81,B11)</f>
         <v/>
       </c>
       <c r="N11" s="4" t="n">
@@ -1206,6 +1207,756 @@
         <v/>
       </c>
       <c r="U11" t="inlineStr">
+        <is>
+          <t>Dynamic INT8 on Linear layers; convolutions stay FP32</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>baseline_fp32</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Baseline: late fusion, softmax attention, FP32</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>138022</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.5434</v>
+      </c>
+      <c r="H12" s="3">
+        <f>AVERAGEIFS(Acc_Runs!D2:D49,Acc_Runs!A2:A49,A12,Acc_Runs!B2:B49,B12)</f>
+        <v/>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>0.01396722353702891</v>
+      </c>
+      <c r="J12" s="3">
+        <f>AVERAGEIFS(Acc_Runs!F2:F49,Acc_Runs!A2:A49,A12,Acc_Runs!B2:B49,B12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="4">
+        <f>AVERAGEIFS(Latency_Runs!E2:E81,Latency_Runs!A2:A81,A12,Latency_Runs!B2:B81,B12)</f>
+        <v/>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>0.2128087622446671</v>
+      </c>
+      <c r="M12" s="4">
+        <f>AVERAGEIFS(Latency_Runs!F2:F81,Latency_Runs!A2:A81,A12,Latency_Runs!B2:B81,B12)</f>
+        <v/>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>0.4549967254243359</v>
+      </c>
+      <c r="O12" t="n">
+        <v>18.945</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="n"/>
+      <c r="S12" s="4" t="n"/>
+      <c r="T12" s="4" t="n"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Reference for the primary device</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>baseline_fp16</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Precision: FP16 weights (GPU only)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>fp16</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>138022</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.2796</v>
+      </c>
+      <c r="H13" s="3">
+        <f>AVERAGEIFS(Acc_Runs!D2:D49,Acc_Runs!A2:A49,A13,Acc_Runs!B2:B49,B13)</f>
+        <v/>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>0.01304160010632646</v>
+      </c>
+      <c r="J13" s="3">
+        <f>AVERAGEIFS(Acc_Runs!F2:F49,Acc_Runs!A2:A49,A13,Acc_Runs!B2:B49,B13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="4">
+        <f>AVERAGEIFS(Latency_Runs!E2:E81,Latency_Runs!A2:A81,A13,Latency_Runs!B2:B81,B13)</f>
+        <v/>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>0.06002445458391568</v>
+      </c>
+      <c r="M13" s="4">
+        <f>AVERAGEIFS(Latency_Runs!F2:F81,Latency_Runs!A2:A81,A13,Latency_Runs!B2:B81,B13)</f>
+        <v/>
+      </c>
+      <c r="N13" s="4" t="n">
+        <v>0.3418055661635718</v>
+      </c>
+      <c r="O13" t="n">
+        <v>18.162</v>
+      </c>
+      <c r="P13" t="n">
+        <v>32.04</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>baseline_fp32</t>
+        </is>
+      </c>
+      <c r="R13" s="3">
+        <f>H13-H12</f>
+        <v/>
+      </c>
+      <c r="S13" s="4">
+        <f>K12/K13</f>
+        <v/>
+      </c>
+      <c r="T13" s="4">
+        <f>G13/G12</f>
+        <v/>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Same weights as baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>linear_attn</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Architecture variant: linear attention</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>138022</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.5434</v>
+      </c>
+      <c r="H14" s="3">
+        <f>AVERAGEIFS(Acc_Runs!D2:D49,Acc_Runs!A2:A49,A14,Acc_Runs!B2:B49,B14)</f>
+        <v/>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>0.0130288142207954</v>
+      </c>
+      <c r="J14" s="3">
+        <f>AVERAGEIFS(Acc_Runs!F2:F49,Acc_Runs!A2:A49,A14,Acc_Runs!B2:B49,B14)</f>
+        <v/>
+      </c>
+      <c r="K14" s="4">
+        <f>AVERAGEIFS(Latency_Runs!E2:E81,Latency_Runs!A2:A81,A14,Latency_Runs!B2:B81,B14)</f>
+        <v/>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>0.3708126568220756</v>
+      </c>
+      <c r="M14" s="4">
+        <f>AVERAGEIFS(Latency_Runs!F2:F81,Latency_Runs!A2:A81,A14,Latency_Runs!B2:B81,B14)</f>
+        <v/>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>0.7766278545253118</v>
+      </c>
+      <c r="O14" t="n">
+        <v>18.945</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>baseline_fp32</t>
+        </is>
+      </c>
+      <c r="R14" s="3">
+        <f>H14-H12</f>
+        <v/>
+      </c>
+      <c r="S14" s="4">
+        <f>K12/K14</f>
+        <v/>
+      </c>
+      <c r="T14" s="4">
+        <f>G14/G12</f>
+        <v/>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Sequence length is only 24: no asymptotic advantage expected</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>early_fusion</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Fusion variant: early fusion, same budget</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>114630</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.4476</v>
+      </c>
+      <c r="H15" s="3">
+        <f>AVERAGEIFS(Acc_Runs!D2:D49,Acc_Runs!A2:A49,A15,Acc_Runs!B2:B49,B15)</f>
+        <v/>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>0.008621678104251716</v>
+      </c>
+      <c r="J15" s="3">
+        <f>AVERAGEIFS(Acc_Runs!F2:F49,Acc_Runs!A2:A49,A15,Acc_Runs!B2:B49,B15)</f>
+        <v/>
+      </c>
+      <c r="K15" s="4">
+        <f>AVERAGEIFS(Latency_Runs!E2:E81,Latency_Runs!A2:A81,A15,Latency_Runs!B2:B81,B15)</f>
+        <v/>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>0.01584599678866139</v>
+      </c>
+      <c r="M15" s="4">
+        <f>AVERAGEIFS(Latency_Runs!F2:F81,Latency_Runs!A2:A81,A15,Latency_Runs!B2:B81,B15)</f>
+        <v/>
+      </c>
+      <c r="N15" s="4" t="n">
+        <v>0.2650769783162325</v>
+      </c>
+      <c r="O15" t="n">
+        <v>19.062</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>baseline_fp32</t>
+        </is>
+      </c>
+      <c r="R15" s="3">
+        <f>H15-H12</f>
+        <v/>
+      </c>
+      <c r="S15" s="4">
+        <f>K12/K15</f>
+        <v/>
+      </c>
+      <c r="T15" s="4">
+        <f>G15/G12</f>
+        <v/>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Image patches + words in one transformer</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>early_fusion_2x</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Fusion variant: early fusion, 2x epochs</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>114630</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.4476</v>
+      </c>
+      <c r="H16" s="3">
+        <f>AVERAGEIFS(Acc_Runs!D2:D49,Acc_Runs!A2:A49,A16,Acc_Runs!B2:B49,B16)</f>
+        <v/>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>0.002645751311064593</v>
+      </c>
+      <c r="J16" s="3">
+        <f>AVERAGEIFS(Acc_Runs!F2:F49,Acc_Runs!A2:A49,A16,Acc_Runs!B2:B49,B16)</f>
+        <v/>
+      </c>
+      <c r="K16" s="4">
+        <f>AVERAGEIFS(Latency_Runs!E2:E81,Latency_Runs!A2:A81,A16,Latency_Runs!B2:B81,B16)</f>
+        <v/>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>0.2440253853728148</v>
+      </c>
+      <c r="M16" s="4">
+        <f>AVERAGEIFS(Latency_Runs!F2:F81,Latency_Runs!A2:A81,A16,Latency_Runs!B2:B81,B16)</f>
+        <v/>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>0.6298405277117195</v>
+      </c>
+      <c r="O16" t="n">
+        <v>19.062</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>baseline_fp32</t>
+        </is>
+      </c>
+      <c r="R16" s="3">
+        <f>H16-H12</f>
+        <v/>
+      </c>
+      <c r="S16" s="4">
+        <f>K12/K16</f>
+        <v/>
+      </c>
+      <c r="T16" s="4">
+        <f>G16/G12</f>
+        <v/>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Same model, double the epochs: separates 'worse' from 'slower to train'</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>student_kd</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Distilled student (KD from baseline)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>9030</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.0467</v>
+      </c>
+      <c r="H17" s="3">
+        <f>AVERAGEIFS(Acc_Runs!D2:D49,Acc_Runs!A2:A49,A17,Acc_Runs!B2:B49,B17)</f>
+        <v/>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>0.01464012750399851</v>
+      </c>
+      <c r="J17" s="3">
+        <f>AVERAGEIFS(Acc_Runs!F2:F49,Acc_Runs!A2:A49,A17,Acc_Runs!B2:B49,B17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="4">
+        <f>AVERAGEIFS(Latency_Runs!E2:E81,Latency_Runs!A2:A81,A17,Latency_Runs!B2:B81,B17)</f>
+        <v/>
+      </c>
+      <c r="L17" s="4" t="n">
+        <v>0.03368797665148789</v>
+      </c>
+      <c r="M17" s="4">
+        <f>AVERAGEIFS(Latency_Runs!F2:F81,Latency_Runs!A2:A81,A17,Latency_Runs!B2:B81,B17)</f>
+        <v/>
+      </c>
+      <c r="N17" s="4" t="n">
+        <v>0.2663248931774851</v>
+      </c>
+      <c r="O17" t="n">
+        <v>18.392</v>
+      </c>
+      <c r="P17" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>baseline_fp32</t>
+        </is>
+      </c>
+      <c r="R17" s="3">
+        <f>H17-H12</f>
+        <v/>
+      </c>
+      <c r="S17" s="4">
+        <f>K12/K17</f>
+        <v/>
+      </c>
+      <c r="T17" s="4">
+        <f>G17/G12</f>
+        <v/>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Width 16, 1 layer, distilled from the baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>student_nokd</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Student, labels only (KD control)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>9030</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.0467</v>
+      </c>
+      <c r="H18" s="3">
+        <f>AVERAGEIFS(Acc_Runs!D2:D49,Acc_Runs!A2:A49,A18,Acc_Runs!B2:B49,B18)</f>
+        <v/>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>0.0072858309981315</v>
+      </c>
+      <c r="J18" s="3">
+        <f>AVERAGEIFS(Acc_Runs!F2:F49,Acc_Runs!A2:A49,A18,Acc_Runs!B2:B49,B18)</f>
+        <v/>
+      </c>
+      <c r="K18" s="4">
+        <f>AVERAGEIFS(Latency_Runs!E2:E81,Latency_Runs!A2:A81,A18,Latency_Runs!B2:B81,B18)</f>
+        <v/>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>0.03428689016045063</v>
+      </c>
+      <c r="M18" s="4">
+        <f>AVERAGEIFS(Latency_Runs!F2:F81,Latency_Runs!A2:A81,A18,Latency_Runs!B2:B81,B18)</f>
+        <v/>
+      </c>
+      <c r="N18" s="4" t="n">
+        <v>0.03483676069781038</v>
+      </c>
+      <c r="O18" t="n">
+        <v>18.392</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>baseline_fp32</t>
+        </is>
+      </c>
+      <c r="R18" s="3">
+        <f>H18-H12</f>
+        <v/>
+      </c>
+      <c r="S18" s="4">
+        <f>K12/K18</f>
+        <v/>
+      </c>
+      <c r="T18" s="4">
+        <f>G18/G12</f>
+        <v/>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Same student from labels only: isolates the effect of KD</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>cpu_baseline_fp32</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Baseline on CPU, FP32</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>138022</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.5427</v>
+      </c>
+      <c r="H19" s="3">
+        <f>AVERAGEIFS(Acc_Runs!D2:D49,Acc_Runs!A2:A49,A19,Acc_Runs!B2:B49,B19)</f>
+        <v/>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>0.01396722353702891</v>
+      </c>
+      <c r="J19" s="3">
+        <f>AVERAGEIFS(Acc_Runs!F2:F49,Acc_Runs!A2:A49,A19,Acc_Runs!B2:B49,B19)</f>
+        <v/>
+      </c>
+      <c r="K19" s="4">
+        <f>AVERAGEIFS(Latency_Runs!E2:E81,Latency_Runs!A2:A81,A19,Latency_Runs!B2:B81,B19)</f>
+        <v/>
+      </c>
+      <c r="L19" s="4" t="n">
+        <v>0.04093921262425083</v>
+      </c>
+      <c r="M19" s="4">
+        <f>AVERAGEIFS(Latency_Runs!F2:F81,Latency_Runs!A2:A81,A19,Latency_Runs!B2:B81,B19)</f>
+        <v/>
+      </c>
+      <c r="N19" s="4" t="n">
+        <v>0.1522348605775018</v>
+      </c>
+      <c r="P19" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R19" s="3" t="n"/>
+      <c r="S19" s="4" t="n"/>
+      <c r="T19" s="4" t="n"/>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>CPU reference when the primary device is a GPU</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>cpu_baseline_int8</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Quantized: dynamic INT8 on CPU</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>int8</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>138022</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.2439</v>
+      </c>
+      <c r="H20" s="3">
+        <f>AVERAGEIFS(Acc_Runs!D2:D49,Acc_Runs!A2:A49,A20,Acc_Runs!B2:B49,B20)</f>
+        <v/>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>0.01331352695569433</v>
+      </c>
+      <c r="J20" s="3">
+        <f>AVERAGEIFS(Acc_Runs!F2:F49,Acc_Runs!A2:A49,A20,Acc_Runs!B2:B49,B20)</f>
+        <v/>
+      </c>
+      <c r="K20" s="4">
+        <f>AVERAGEIFS(Latency_Runs!E2:E81,Latency_Runs!A2:A81,A20,Latency_Runs!B2:B81,B20)</f>
+        <v/>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>1.012911694167388</v>
+      </c>
+      <c r="M20" s="4">
+        <f>AVERAGEIFS(Latency_Runs!F2:F81,Latency_Runs!A2:A81,A20,Latency_Runs!B2:B81,B20)</f>
+        <v/>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>4.991442112596982</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>cpu_baseline_fp32</t>
+        </is>
+      </c>
+      <c r="R20" s="3">
+        <f>H20-H19</f>
+        <v/>
+      </c>
+      <c r="S20" s="4">
+        <f>K19/K20</f>
+        <v/>
+      </c>
+      <c r="T20" s="4">
+        <f>G20/G19</f>
+        <v/>
+      </c>
+      <c r="U20" t="inlineStr">
         <is>
           <t>Dynamic INT8 on Linear layers; convolutions stay FP32</t>
         </is>
@@ -1382,7 +2133,441 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:K12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="33" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Same code, same seeds, same budgets: Intel VM (tag cpu) vs Colab / T4 GPU (tag t4gpu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>config</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>VM acc</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>GPU-run acc</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>acc diff</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>VM p50 ms</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>GPU-run p50 ms</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>p50 speedup (VM / GPU run)</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>VM p95 ms</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>GPU-run p95 ms</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>p95 speedup</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>where the GPU run executed it</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>baseline_fp32</t>
+        </is>
+      </c>
+      <c r="B4" s="3">
+        <f>Board!H5</f>
+        <v/>
+      </c>
+      <c r="C4" s="3">
+        <f>Board!H12</f>
+        <v/>
+      </c>
+      <c r="D4" s="3">
+        <f>C4-B4</f>
+        <v/>
+      </c>
+      <c r="E4" s="4">
+        <f>Board!K5</f>
+        <v/>
+      </c>
+      <c r="F4" s="4">
+        <f>Board!K12</f>
+        <v/>
+      </c>
+      <c r="G4" s="4">
+        <f>E4/F4</f>
+        <v/>
+      </c>
+      <c r="H4" s="4">
+        <f>Board!M5</f>
+        <v/>
+      </c>
+      <c r="I4" s="4">
+        <f>Board!M12</f>
+        <v/>
+      </c>
+      <c r="J4" s="4">
+        <f>H4/I4</f>
+        <v/>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>linear_attn</t>
+        </is>
+      </c>
+      <c r="B5" s="3">
+        <f>Board!H6</f>
+        <v/>
+      </c>
+      <c r="C5" s="3">
+        <f>Board!H14</f>
+        <v/>
+      </c>
+      <c r="D5" s="3">
+        <f>C5-B5</f>
+        <v/>
+      </c>
+      <c r="E5" s="4">
+        <f>Board!K6</f>
+        <v/>
+      </c>
+      <c r="F5" s="4">
+        <f>Board!K14</f>
+        <v/>
+      </c>
+      <c r="G5" s="4">
+        <f>E5/F5</f>
+        <v/>
+      </c>
+      <c r="H5" s="4">
+        <f>Board!M6</f>
+        <v/>
+      </c>
+      <c r="I5" s="4">
+        <f>Board!M14</f>
+        <v/>
+      </c>
+      <c r="J5" s="4">
+        <f>H5/I5</f>
+        <v/>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>early_fusion</t>
+        </is>
+      </c>
+      <c r="B6" s="3">
+        <f>Board!H7</f>
+        <v/>
+      </c>
+      <c r="C6" s="3">
+        <f>Board!H15</f>
+        <v/>
+      </c>
+      <c r="D6" s="3">
+        <f>C6-B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="4">
+        <f>Board!K7</f>
+        <v/>
+      </c>
+      <c r="F6" s="4">
+        <f>Board!K15</f>
+        <v/>
+      </c>
+      <c r="G6" s="4">
+        <f>E6/F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="4">
+        <f>Board!M7</f>
+        <v/>
+      </c>
+      <c r="I6" s="4">
+        <f>Board!M15</f>
+        <v/>
+      </c>
+      <c r="J6" s="4">
+        <f>H6/I6</f>
+        <v/>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>early_fusion_2x</t>
+        </is>
+      </c>
+      <c r="B7" s="3">
+        <f>Board!H8</f>
+        <v/>
+      </c>
+      <c r="C7" s="3">
+        <f>Board!H16</f>
+        <v/>
+      </c>
+      <c r="D7" s="3">
+        <f>C7-B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="4">
+        <f>Board!K8</f>
+        <v/>
+      </c>
+      <c r="F7" s="4">
+        <f>Board!K16</f>
+        <v/>
+      </c>
+      <c r="G7" s="4">
+        <f>E7/F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="4">
+        <f>Board!M8</f>
+        <v/>
+      </c>
+      <c r="I7" s="4">
+        <f>Board!M16</f>
+        <v/>
+      </c>
+      <c r="J7" s="4">
+        <f>H7/I7</f>
+        <v/>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>student_kd</t>
+        </is>
+      </c>
+      <c r="B8" s="3">
+        <f>Board!H9</f>
+        <v/>
+      </c>
+      <c r="C8" s="3">
+        <f>Board!H17</f>
+        <v/>
+      </c>
+      <c r="D8" s="3">
+        <f>C8-B8</f>
+        <v/>
+      </c>
+      <c r="E8" s="4">
+        <f>Board!K9</f>
+        <v/>
+      </c>
+      <c r="F8" s="4">
+        <f>Board!K17</f>
+        <v/>
+      </c>
+      <c r="G8" s="4">
+        <f>E8/F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="4">
+        <f>Board!M9</f>
+        <v/>
+      </c>
+      <c r="I8" s="4">
+        <f>Board!M17</f>
+        <v/>
+      </c>
+      <c r="J8" s="4">
+        <f>H8/I8</f>
+        <v/>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>student_nokd</t>
+        </is>
+      </c>
+      <c r="B9" s="3">
+        <f>Board!H10</f>
+        <v/>
+      </c>
+      <c r="C9" s="3">
+        <f>Board!H18</f>
+        <v/>
+      </c>
+      <c r="D9" s="3">
+        <f>C9-B9</f>
+        <v/>
+      </c>
+      <c r="E9" s="4">
+        <f>Board!K10</f>
+        <v/>
+      </c>
+      <c r="F9" s="4">
+        <f>Board!K18</f>
+        <v/>
+      </c>
+      <c r="G9" s="4">
+        <f>E9/F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="4">
+        <f>Board!M10</f>
+        <v/>
+      </c>
+      <c r="I9" s="4">
+        <f>Board!M18</f>
+        <v/>
+      </c>
+      <c r="J9" s="4">
+        <f>H9/I9</f>
+        <v/>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>cpu_baseline_int8</t>
+        </is>
+      </c>
+      <c r="B10" s="3">
+        <f>Board!H11</f>
+        <v/>
+      </c>
+      <c r="C10" s="3">
+        <f>Board!H20</f>
+        <v/>
+      </c>
+      <c r="D10" s="3">
+        <f>C10-B10</f>
+        <v/>
+      </c>
+      <c r="E10" s="4">
+        <f>Board!K11</f>
+        <v/>
+      </c>
+      <c r="F10" s="4">
+        <f>Board!K20</f>
+        <v/>
+      </c>
+      <c r="G10" s="4">
+        <f>E10/F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="4">
+        <f>Board!M11</f>
+        <v/>
+      </c>
+      <c r="I10" s="4">
+        <f>Board!M20</f>
+        <v/>
+      </c>
+      <c r="J10" s="4">
+        <f>H10/I10</f>
+        <v/>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Quality should agree across hardware (small drift = floating-point order). Latency is what the hardware changes. Note the INT8 and CPU rows run on the CPU of whichever machine this was: the T4 run's CPU is Colab's 2-vCPU Xeon, not the T4.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1929,18 +3114,666 @@
         <v>0.0174480599208049</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>baseline_fp32</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.7775</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.0182287244479694</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>baseline_fp16</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.7775</v>
+      </c>
+      <c r="E24" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.0182287244479694</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>linear_attn</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.7795</v>
+      </c>
+      <c r="E25" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.0181699373636785</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>early_fusion</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.286</v>
+      </c>
+      <c r="E26" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.0198049247208869</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>early_fusion_2x</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.2715</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.0194912983200196</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>student_kd</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.737</v>
+      </c>
+      <c r="E28" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.0192953513779873</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>student_nokd</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="E29" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.0194800237987534</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>cpu_baseline_fp32</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.7775</v>
+      </c>
+      <c r="E30" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.0182287244479694</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>cpu_baseline_int8</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.0182140850113312</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>baseline_fp32</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.7955</v>
+      </c>
+      <c r="E32" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.0176769698704274</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>baseline_fp16</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.795</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.0176930037020286</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>linear_attn</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0.794</v>
+      </c>
+      <c r="E34" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.0177249465781987</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>early_fusion</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0.292</v>
+      </c>
+      <c r="E35" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.0199273306993184</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>early_fusion_2x</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0.2765</v>
+      </c>
+      <c r="E36" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.0196023396103628</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>student_kd</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0.766</v>
+      </c>
+      <c r="E37" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.0185551037507204</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>student_nokd</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0.7435</v>
+      </c>
+      <c r="E38" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.0191392645156495</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>cpu_baseline_fp32</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0.7955</v>
+      </c>
+      <c r="E39" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.0176769698704274</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>cpu_baseline_int8</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.7935</v>
+      </c>
+      <c r="E40" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.0177408558474499</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>baseline_fp32</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.805</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.0173642615737036</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>baseline_fp16</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>2</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0.803</v>
+      </c>
+      <c r="E42" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.0174313875752907</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>linear_attn</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0.8055</v>
+      </c>
+      <c r="E43" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.0173473702848587</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>early_fusion</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>2</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0.303</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.0201408955312319</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>early_fusion_2x</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0.2755</v>
+      </c>
+      <c r="E45" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.0195803779279154</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>student_kd</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>2</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0.755</v>
+      </c>
+      <c r="E46" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.0188494026430547</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>student_nokd</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0.735</v>
+      </c>
+      <c r="E47" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.0193422806307839</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>cpu_baseline_fp32</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0.805</v>
+      </c>
+      <c r="E48" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.0173642615737036</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>cpu_baseline_int8</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>2</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0.8045</v>
+      </c>
+      <c r="E49" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.0173811088196351</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3226,12 +5059,1587 @@
         <v>300</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>cpu_baseline_fp32</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>1.618636000102924</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1.978295350124881</v>
+      </c>
+      <c r="G37" t="n">
+        <v>1.685564606671808</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0.2797914858190699</v>
+      </c>
+      <c r="I37" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>student_kd</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>1.089445000047817</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1.260078050120228</v>
+      </c>
+      <c r="G38" t="n">
+        <v>1.113038440001522</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.0864609058619993</v>
+      </c>
+      <c r="I38" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>baseline_fp16</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>1.534547000119346</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1.76129835001575</v>
+      </c>
+      <c r="G39" t="n">
+        <v>1.571717823330043</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.1096128282055493</v>
+      </c>
+      <c r="I39" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>early_fusion</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1.180277000116803</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1.529318500001864</v>
+      </c>
+      <c r="G40" t="n">
+        <v>1.218986350004343</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0.1422045276002684</v>
+      </c>
+      <c r="I40" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>early_fusion_2x</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
+        <v>1.168583999969996</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1.695740749948983</v>
+      </c>
+      <c r="G41" t="n">
+        <v>1.241200779992748</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.2012579923644287</v>
+      </c>
+      <c r="I41" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>linear_attn</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" t="n">
+        <v>2.668060499900093</v>
+      </c>
+      <c r="F42" t="n">
+        <v>3.39109559993176</v>
+      </c>
+      <c r="G42" t="n">
+        <v>2.760056880000926</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0.3396365981080261</v>
+      </c>
+      <c r="I42" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>baseline_fp32</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="n">
+        <v>1.560408500040467</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1.878316050010654</v>
+      </c>
+      <c r="G43" t="n">
+        <v>1.60470053666586</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.17635201400297</v>
+      </c>
+      <c r="I43" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>cpu_baseline_int8</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2.158507499984808</v>
+      </c>
+      <c r="F44" t="n">
+        <v>2.542608299916083</v>
+      </c>
+      <c r="G44" t="n">
+        <v>2.262441819998457</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.5735702614926508</v>
+      </c>
+      <c r="I44" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>student_nokd</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>1.164403499956279</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1.299103699932402</v>
+      </c>
+      <c r="G45" t="n">
+        <v>1.176085939999514</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.1063794077109101</v>
+      </c>
+      <c r="I45" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>linear_attn</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" t="n">
+        <v>2.633702000139237</v>
+      </c>
+      <c r="F46" t="n">
+        <v>3.115899400029321</v>
+      </c>
+      <c r="G46" t="n">
+        <v>2.671164576667404</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.2730803356191356</v>
+      </c>
+      <c r="I46" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>baseline_fp32</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" t="n">
+        <v>1.50731849987551</v>
+      </c>
+      <c r="F47" t="n">
+        <v>1.977252399956344</v>
+      </c>
+      <c r="G47" t="n">
+        <v>1.558759256668054</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0.2251977247695167</v>
+      </c>
+      <c r="I47" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>early_fusion</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" t="n">
+        <v>1.203610000061417</v>
+      </c>
+      <c r="F48" t="n">
+        <v>1.996345150155321</v>
+      </c>
+      <c r="G48" t="n">
+        <v>1.296255429996715</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0.2960699986380846</v>
+      </c>
+      <c r="I48" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>cpu_baseline_int8</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" t="n">
+        <v>4.463238500079569</v>
+      </c>
+      <c r="F49" t="n">
+        <v>13.76187190014662</v>
+      </c>
+      <c r="G49" t="n">
+        <v>7.937830530008796</v>
+      </c>
+      <c r="H49" t="n">
+        <v>16.98800946192435</v>
+      </c>
+      <c r="I49" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>student_nokd</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" t="n">
+        <v>1.087420999965616</v>
+      </c>
+      <c r="F50" t="n">
+        <v>1.277315600009388</v>
+      </c>
+      <c r="G50" t="n">
+        <v>1.117704739999681</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0.0810843499801195</v>
+      </c>
+      <c r="I50" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>baseline_fp16</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" t="n">
+        <v>1.650184499908391</v>
+      </c>
+      <c r="F51" t="n">
+        <v>2.421268900127416</v>
+      </c>
+      <c r="G51" t="n">
+        <v>1.722757676670123</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0.2609472524365014</v>
+      </c>
+      <c r="I51" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>early_fusion_2x</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" t="n">
+        <v>1.214341000036256</v>
+      </c>
+      <c r="F52" t="n">
+        <v>1.394826050113807</v>
+      </c>
+      <c r="G52" t="n">
+        <v>1.236991953339839</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0.1027369079627979</v>
+      </c>
+      <c r="I52" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>student_kd</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" t="n">
+        <v>1.163632499924461</v>
+      </c>
+      <c r="F53" t="n">
+        <v>1.791790600100285</v>
+      </c>
+      <c r="G53" t="n">
+        <v>1.217338996663481</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0.1987905779326592</v>
+      </c>
+      <c r="I53" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>cpu_baseline_fp32</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" t="n">
+        <v>1.681148499983465</v>
+      </c>
+      <c r="F54" t="n">
+        <v>1.94976875014845</v>
+      </c>
+      <c r="G54" t="n">
+        <v>1.703658660001868</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0.166358057125721</v>
+      </c>
+      <c r="I54" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>linear_attn</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>2</v>
+      </c>
+      <c r="E55" t="n">
+        <v>2.597155999978895</v>
+      </c>
+      <c r="F55" t="n">
+        <v>3.409377450134345</v>
+      </c>
+      <c r="G55" t="n">
+        <v>2.686109560006571</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0.3602118957422078</v>
+      </c>
+      <c r="I55" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>baseline_fp32</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>2</v>
+      </c>
+      <c r="E56" t="n">
+        <v>1.516178499969101</v>
+      </c>
+      <c r="F56" t="n">
+        <v>2.31350145010083</v>
+      </c>
+      <c r="G56" t="n">
+        <v>1.595011769999625</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0.319942361501585</v>
+      </c>
+      <c r="I56" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>early_fusion</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>2</v>
+      </c>
+      <c r="E57" t="n">
+        <v>1.215032999994037</v>
+      </c>
+      <c r="F57" t="n">
+        <v>1.431135500001801</v>
+      </c>
+      <c r="G57" t="n">
+        <v>1.232954860001882</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0.1061238530034182</v>
+      </c>
+      <c r="I57" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>cpu_baseline_int8</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>2</v>
+      </c>
+      <c r="E58" t="n">
+        <v>2.241324999999961</v>
+      </c>
+      <c r="F58" t="n">
+        <v>2.812533949997942</v>
+      </c>
+      <c r="G58" t="n">
+        <v>2.367362453330012</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0.7458944318190532</v>
+      </c>
+      <c r="I58" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>student_nokd</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>2</v>
+      </c>
+      <c r="E59" t="n">
+        <v>1.175529999954961</v>
+      </c>
+      <c r="F59" t="n">
+        <v>1.36960315013539</v>
+      </c>
+      <c r="G59" t="n">
+        <v>1.202908483336766</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0.1145181578689272</v>
+      </c>
+      <c r="I59" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>student_kd</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>2</v>
+      </c>
+      <c r="E60" t="n">
+        <v>1.176713499944526</v>
+      </c>
+      <c r="F60" t="n">
+        <v>1.864269250029338</v>
+      </c>
+      <c r="G60" t="n">
+        <v>1.267625580000337</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0.246883842799664</v>
+      </c>
+      <c r="I60" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>cpu_baseline_fp32</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>2</v>
+      </c>
+      <c r="E61" t="n">
+        <v>1.668630999915877</v>
+      </c>
+      <c r="F61" t="n">
+        <v>1.971609100019123</v>
+      </c>
+      <c r="G61" t="n">
+        <v>1.700621120002476</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0.1534869785702583</v>
+      </c>
+      <c r="I61" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>early_fusion_2x</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>2</v>
+      </c>
+      <c r="E62" t="n">
+        <v>1.235564500007058</v>
+      </c>
+      <c r="F62" t="n">
+        <v>1.900117250045241</v>
+      </c>
+      <c r="G62" t="n">
+        <v>1.298906449997806</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0.206731868589817</v>
+      </c>
+      <c r="I62" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>baseline_fp16</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>2</v>
+      </c>
+      <c r="E63" t="n">
+        <v>1.65401850017588</v>
+      </c>
+      <c r="F63" t="n">
+        <v>1.881457599870373</v>
+      </c>
+      <c r="G63" t="n">
+        <v>1.669664219994047</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0.1016004993883821</v>
+      </c>
+      <c r="I63" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>cpu_baseline_fp32</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>3</v>
+      </c>
+      <c r="E64" t="n">
+        <v>1.733302999923581</v>
+      </c>
+      <c r="F64" t="n">
+        <v>2.31281664995322</v>
+      </c>
+      <c r="G64" t="n">
+        <v>1.857239853334249</v>
+      </c>
+      <c r="H64" t="n">
+        <v>0.5877003674176515</v>
+      </c>
+      <c r="I64" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>student_nokd</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>3</v>
+      </c>
+      <c r="E65" t="n">
+        <v>1.151327499997024</v>
+      </c>
+      <c r="F65" t="n">
+        <v>1.327098700016904</v>
+      </c>
+      <c r="G65" t="n">
+        <v>1.1670959499952</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0.0927031449064166</v>
+      </c>
+      <c r="I65" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>cpu_baseline_int8</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>3</v>
+      </c>
+      <c r="E66" t="n">
+        <v>2.197499499970945</v>
+      </c>
+      <c r="F66" t="n">
+        <v>2.551064449994557</v>
+      </c>
+      <c r="G66" t="n">
+        <v>2.288223746665305</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0.6029234590241304</v>
+      </c>
+      <c r="I66" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>linear_attn</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>3</v>
+      </c>
+      <c r="E67" t="n">
+        <v>3.460898500065923</v>
+      </c>
+      <c r="F67" t="n">
+        <v>5.03900405000195</v>
+      </c>
+      <c r="G67" t="n">
+        <v>3.602061383339787</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0.7231082953029945</v>
+      </c>
+      <c r="I67" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>baseline_fp32</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>3</v>
+      </c>
+      <c r="E68" t="n">
+        <v>1.994294500036631</v>
+      </c>
+      <c r="F68" t="n">
+        <v>2.968314449913124</v>
+      </c>
+      <c r="G68" t="n">
+        <v>2.146614879990617</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0.4256569378137076</v>
+      </c>
+      <c r="I68" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>early_fusion_2x</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>3</v>
+      </c>
+      <c r="E69" t="n">
+        <v>1.75299400007134</v>
+      </c>
+      <c r="F69" t="n">
+        <v>2.94512894994341</v>
+      </c>
+      <c r="G69" t="n">
+        <v>1.907252760002697</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0.4886451753525205</v>
+      </c>
+      <c r="I69" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>early_fusion</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>3</v>
+      </c>
+      <c r="E70" t="n">
+        <v>1.180649500042818</v>
+      </c>
+      <c r="F70" t="n">
+        <v>1.909582050018344</v>
+      </c>
+      <c r="G70" t="n">
+        <v>1.258716943334548</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0.2452578911835516</v>
+      </c>
+      <c r="I70" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>student_kd</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>3</v>
+      </c>
+      <c r="E71" t="n">
+        <v>1.155330500068885</v>
+      </c>
+      <c r="F71" t="n">
+        <v>1.36836549996815</v>
+      </c>
+      <c r="G71" t="n">
+        <v>1.178440366667625</v>
+      </c>
+      <c r="H71" t="n">
+        <v>0.117263759483408</v>
+      </c>
+      <c r="I71" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>baseline_fp16</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>3</v>
+      </c>
+      <c r="E72" t="n">
+        <v>1.68290400006299</v>
+      </c>
+      <c r="F72" t="n">
+        <v>2.003191350024737</v>
+      </c>
+      <c r="G72" t="n">
+        <v>1.738235216671455</v>
+      </c>
+      <c r="H72" t="n">
+        <v>0.2440795530129506</v>
+      </c>
+      <c r="I72" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>baseline_fp16</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>4</v>
+      </c>
+      <c r="E73" t="n">
+        <v>1.673974000027556</v>
+      </c>
+      <c r="F73" t="n">
+        <v>2.541143199994167</v>
+      </c>
+      <c r="G73" t="n">
+        <v>1.756235346677689</v>
+      </c>
+      <c r="H73" t="n">
+        <v>0.2686199989369976</v>
+      </c>
+      <c r="I73" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>student_nokd</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>4</v>
+      </c>
+      <c r="E74" t="n">
+        <v>1.137702499931947</v>
+      </c>
+      <c r="F74" t="n">
+        <v>1.329277549871222</v>
+      </c>
+      <c r="G74" t="n">
+        <v>1.151863480002551</v>
+      </c>
+      <c r="H74" t="n">
+        <v>0.0969718027250825</v>
+      </c>
+      <c r="I74" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>student_kd</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>4</v>
+      </c>
+      <c r="E75" t="n">
+        <v>1.145958000051905</v>
+      </c>
+      <c r="F75" t="n">
+        <v>1.45266004997211</v>
+      </c>
+      <c r="G75" t="n">
+        <v>1.169393706669174</v>
+      </c>
+      <c r="H75" t="n">
+        <v>0.1269890707248863</v>
+      </c>
+      <c r="I75" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>baseline_fp32</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>4</v>
+      </c>
+      <c r="E76" t="n">
+        <v>1.501207999922372</v>
+      </c>
+      <c r="F76" t="n">
+        <v>1.930336199984595</v>
+      </c>
+      <c r="G76" t="n">
+        <v>1.557402026664931</v>
+      </c>
+      <c r="H76" t="n">
+        <v>0.2255041373563886</v>
+      </c>
+      <c r="I76" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>linear_attn</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>4</v>
+      </c>
+      <c r="E77" t="n">
+        <v>2.635632499959684</v>
+      </c>
+      <c r="F77" t="n">
+        <v>3.3771640000964</v>
+      </c>
+      <c r="G77" t="n">
+        <v>2.72471246666934</v>
+      </c>
+      <c r="H77" t="n">
+        <v>0.3300400449921181</v>
+      </c>
+      <c r="I77" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>early_fusion_2x</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>4</v>
+      </c>
+      <c r="E78" t="n">
+        <v>1.222547999873314</v>
+      </c>
+      <c r="F78" t="n">
+        <v>1.452714300114621</v>
+      </c>
+      <c r="G78" t="n">
+        <v>1.253842903333862</v>
+      </c>
+      <c r="H78" t="n">
+        <v>0.1344359530893431</v>
+      </c>
+      <c r="I78" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>cpu_baseline_int8</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>4</v>
+      </c>
+      <c r="E79" t="n">
+        <v>2.199655000026723</v>
+      </c>
+      <c r="F79" t="n">
+        <v>2.509672750045411</v>
+      </c>
+      <c r="G79" t="n">
+        <v>2.293766746656729</v>
+      </c>
+      <c r="H79" t="n">
+        <v>0.6669677884697121</v>
+      </c>
+      <c r="I79" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>cpu_baseline_fp32</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>cpu</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>4</v>
+      </c>
+      <c r="E80" t="n">
+        <v>1.683359499907056</v>
+      </c>
+      <c r="F80" t="n">
+        <v>1.999094399980095</v>
+      </c>
+      <c r="G80" t="n">
+        <v>1.779198429994722</v>
+      </c>
+      <c r="H80" t="n">
+        <v>0.5666829893281655</v>
+      </c>
+      <c r="I80" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>early_fusion</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>4</v>
+      </c>
+      <c r="E81" t="n">
+        <v>1.206418000037956</v>
+      </c>
+      <c r="F81" t="n">
+        <v>1.469109300046512</v>
+      </c>
+      <c r="G81" t="n">
+        <v>1.232111806665822</v>
+      </c>
+      <c r="H81" t="n">
+        <v>0.133990490052849</v>
+      </c>
+      <c r="I81" t="n">
+        <v>300</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3855,17 +7263,18 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3879,6 +7288,11 @@
           <t>cpu</t>
         </is>
       </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>t4gpu</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3891,6 +7305,11 @@
           <t>intel-vm</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>colab-t4</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3903,6 +7322,11 @@
           <t>Intel VM (CPU only)</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Colab (T4 GPU)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3915,6 +7339,11 @@
           <t>windows</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>colab</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3927,6 +7356,11 @@
           <t>3.14.7</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>3.13.15</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3939,6 +7373,11 @@
           <t>2.14.1+cpu</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2.11.0+cu130</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3951,6 +7390,11 @@
           <t>None</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>13.0</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3963,6 +7407,11 @@
           <t>cpu</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>cuda</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3975,6 +7424,11 @@
           <t>None</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3987,6 +7441,11 @@
           <t>None</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>14.6</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3999,6 +7458,11 @@
           <t>None</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>7.5</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4011,6 +7475,11 @@
           <t>None</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>580.82.07</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4023,6 +7492,11 @@
           <t>13th Gen Intel(R) Core(TM) i9-13900HX</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Intel(R) Xeon(R) CPU @ 2.00GHz</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4035,6 +7509,11 @@
           <t>16</t>
         </is>
       </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4047,6 +7526,11 @@
           <t>8.5</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>12.7</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4059,6 +7543,11 @@
           <t>True</t>
         </is>
       </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4071,6 +7560,11 @@
           <t>Virtual Machine</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Google Compute Engine (docker)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4083,6 +7577,11 @@
           <t>2.5.4</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2.1.3</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4095,6 +7594,11 @@
           <t>3.0.6</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2.2.3</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4107,6 +7611,11 @@
           <t>3.11.2</t>
         </is>
       </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>3.10.0</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4116,6 +7625,9 @@
       </c>
       <c r="B22" t="n">
         <v>1177.5</v>
+      </c>
+      <c r="C22" t="n">
+        <v>302.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>